<commit_message>
Update model outputs 2026-06-11 20:49:54
</commit_message>
<xml_diff>
--- a/files/NRL_upcoming_projections.xlsx
+++ b/files/NRL_upcoming_projections.xlsx
@@ -644,16 +644,16 @@
         <v>49.5</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>-9.86</v>
+        <v>-6.49</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>47.12</v>
+        <v>50.72</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>-0.7</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>47.33</v>
+        <v>50.61</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>30</v>
@@ -671,7 +671,7 @@
         <v>0</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>-0.29</v>
+        <v>-0.3</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>4.07</v>
@@ -718,16 +718,16 @@
         <v>49.5</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>-9.83</v>
+        <v>-6.47</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>46.2</v>
+        <v>49.79</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>-0.7</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>47.33</v>
+        <v>50.61</v>
       </c>
       <c r="Q3" s="3" t="s">
         <v>30</v>
@@ -745,13 +745,13 @@
         <v>-0.02</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>-0.29</v>
+        <v>-0.3</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>4.07</v>
       </c>
       <c r="X3" s="4" t="n">
-        <v>-0.92</v>
+        <v>-0.93</v>
       </c>
     </row>
     <row r="4">
@@ -792,16 +792,16 @@
         <v>49.5</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>-4.93</v>
+        <v>-3.25</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>23.56</v>
+        <v>25.36</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>-0.35</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>23.67</v>
+        <v>25.3</v>
       </c>
       <c r="Q4" s="3" t="s">
         <v>30</v>
@@ -866,16 +866,16 @@
         <v>49.5</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>-4.92</v>
+        <v>-3.23</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>23.1</v>
+        <v>24.9</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>-0.35</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>23.67</v>
+        <v>25.3</v>
       </c>
       <c r="Q5" s="3" t="s">
         <v>30</v>
@@ -940,16 +940,16 @@
         <v>51</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>-6.14</v>
+        <v>-0.21</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>46.03</v>
+        <v>49.67</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>-1.86</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>44.59</v>
+        <v>47.87</v>
       </c>
       <c r="Q6" s="3" t="s">
         <v>30</v>
@@ -967,7 +967,7 @@
         <v>0</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>-0.56</v>
+        <v>-0.57</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>4.07</v>
@@ -1014,16 +1014,16 @@
         <v>51</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>-6.05</v>
+        <v>-0.13</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>43.96</v>
+        <v>47.58</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>-1.86</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>44.59</v>
+        <v>47.87</v>
       </c>
       <c r="Q7" s="3" t="s">
         <v>30</v>
@@ -1041,13 +1041,13 @@
         <v>-0.08</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>-0.56</v>
+        <v>-0.57</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>4.07</v>
       </c>
       <c r="X7" s="4" t="n">
-        <v>-2.07</v>
+        <v>-2.09</v>
       </c>
     </row>
     <row r="8">
@@ -1088,16 +1088,16 @@
         <v>51</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>-3.07</v>
+        <v>-0.11</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>23.02</v>
+        <v>24.84</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>-0.93</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>22.3</v>
+        <v>23.94</v>
       </c>
       <c r="Q8" s="3" t="s">
         <v>30</v>
@@ -1162,16 +1162,16 @@
         <v>51</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>-3.03</v>
+        <v>-0.06</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>21.98</v>
+        <v>23.79</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>-0.93</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>22.3</v>
+        <v>23.94</v>
       </c>
       <c r="Q9" s="3" t="s">
         <v>30</v>
@@ -1224,7 +1224,7 @@
         <v>29</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>1</v>
@@ -1236,16 +1236,16 @@
         <v>49</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2.16</v>
+        <v>-1.89</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>46.61</v>
+        <v>50.2</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>2.52</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>47.22</v>
+        <v>50.5</v>
       </c>
       <c r="Q10" s="3" t="s">
         <v>30</v>
@@ -1298,7 +1298,7 @@
         <v>31</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11" s="5" t="n">
         <v>1</v>
@@ -1310,16 +1310,16 @@
         <v>49</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>2.16</v>
+        <v>-1.89</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>46.61</v>
+        <v>50.2</v>
       </c>
       <c r="O11" s="4" t="n">
         <v>2.52</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>47.22</v>
+        <v>50.5</v>
       </c>
       <c r="Q11" s="3" t="s">
         <v>30</v>
@@ -1372,7 +1372,7 @@
         <v>29</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>1</v>
@@ -1384,16 +1384,16 @@
         <v>49</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>1.08</v>
+        <v>-0.95</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>23.31</v>
+        <v>25.1</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>1.26</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>23.61</v>
+        <v>25.25</v>
       </c>
       <c r="Q12" s="3" t="s">
         <v>30</v>
@@ -1446,7 +1446,7 @@
         <v>31</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" s="5" t="n">
         <v>1</v>
@@ -1458,16 +1458,16 @@
         <v>49</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>1.08</v>
+        <v>-0.95</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>23.31</v>
+        <v>25.1</v>
       </c>
       <c r="O13" s="4" t="n">
         <v>1.26</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>23.61</v>
+        <v>25.25</v>
       </c>
       <c r="Q13" s="3" t="s">
         <v>30</v>
@@ -1532,16 +1532,16 @@
         <v>49.5</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>-2.56</v>
+        <v>-0.18</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>47.17</v>
+        <v>50.62</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>-0.72</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>47.88</v>
+        <v>51.15</v>
       </c>
       <c r="Q14" s="3" t="s">
         <v>30</v>
@@ -1606,16 +1606,16 @@
         <v>49.5</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>-2.56</v>
+        <v>-0.18</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>47.17</v>
+        <v>50.62</v>
       </c>
       <c r="O15" s="4" t="n">
         <v>-0.72</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>47.88</v>
+        <v>51.15</v>
       </c>
       <c r="Q15" s="3" t="s">
         <v>30</v>
@@ -1680,16 +1680,16 @@
         <v>49.5</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>-1.28</v>
+        <v>-0.09</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>23.58</v>
+        <v>25.31</v>
       </c>
       <c r="O16" s="4" t="n">
         <v>-0.36</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>23.94</v>
+        <v>25.58</v>
       </c>
       <c r="Q16" s="3" t="s">
         <v>30</v>
@@ -1754,16 +1754,16 @@
         <v>49.5</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>-1.28</v>
+        <v>-0.09</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>23.58</v>
+        <v>25.31</v>
       </c>
       <c r="O17" s="4" t="n">
         <v>-0.36</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>23.94</v>
+        <v>25.58</v>
       </c>
       <c r="Q17" s="3" t="s">
         <v>30</v>
@@ -1828,16 +1828,16 @@
         <v>50.5</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>-2.77</v>
+        <v>-4.44</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>49.47</v>
+        <v>53.18</v>
       </c>
       <c r="O18" s="4" t="n">
         <v>-2.97</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>49.87</v>
+        <v>53.15</v>
       </c>
       <c r="Q18" s="3" t="s">
         <v>30</v>
@@ -1855,7 +1855,7 @@
         <v>0</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>1.95</v>
+        <v>1.98</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>4.07</v>
@@ -1902,16 +1902,16 @@
         <v>50.5</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>-2.75</v>
+        <v>-4.42</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>48.77</v>
+        <v>52.47</v>
       </c>
       <c r="O19" s="4" t="n">
         <v>-2.97</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>49.87</v>
+        <v>53.15</v>
       </c>
       <c r="Q19" s="3" t="s">
         <v>30</v>
@@ -1929,7 +1929,7 @@
         <v>-0.02</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>1.95</v>
+        <v>1.98</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>4.07</v>
@@ -1976,16 +1976,16 @@
         <v>50.5</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>-1.38</v>
+        <v>-2.22</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>24.73</v>
+        <v>26.59</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>-1.49</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>24.94</v>
+        <v>26.57</v>
       </c>
       <c r="Q20" s="3" t="s">
         <v>30</v>
@@ -2003,7 +2003,7 @@
         <v>0</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>2.04</v>
@@ -2050,16 +2050,16 @@
         <v>50.5</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>-1.38</v>
+        <v>-2.21</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>24.39</v>
+        <v>26.24</v>
       </c>
       <c r="O21" s="4" t="n">
         <v>-1.49</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>24.94</v>
+        <v>26.57</v>
       </c>
       <c r="Q21" s="3" t="s">
         <v>30</v>
@@ -2077,7 +2077,7 @@
         <v>-0.01</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>2.04</v>

</xml_diff>

<commit_message>
Update model outputs 2026-06-23 19:57:18
</commit_message>
<xml_diff>
--- a/files/NRL_upcoming_projections.xlsx
+++ b/files/NRL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -86,118 +86,124 @@
     <t xml:space="preserve">Rain Total Adj</t>
   </si>
   <si>
+    <t xml:space="preserve">Home Raw Form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away Raw Form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net Uncapped Form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parramatta eels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">south sydney rabbitohs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CommBank Stadium, Sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">same_city_different_ground</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast titans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">canterbury-bankstown bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cbus Super Stadium, Gold Coast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diff_city</t>
+  </si>
+  <si>
     <t xml:space="preserve">20:00</t>
   </si>
   <si>
+    <t xml:space="preserve">brisbane broncos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney roosters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suncorp Stadium, Brisbane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dolphins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">warriors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north queensland cowboys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">penrith panthers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Queensland Country Bank Stadium, Townsville</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">manly-warringah sea eagles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne storm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 Pines Park, Sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">canberra raiders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st george-illawarra dragons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GIO Stadium, Canberra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:05</t>
+  </si>
+  <si>
     <t xml:space="preserve">newcastle knights</t>
   </si>
   <si>
-    <t xml:space="preserve">st george-illawarra dragons</t>
+    <t xml:space="preserve">wests tigers</t>
   </si>
   <si>
     <t xml:space="preserve">McDonald Jones Stadium, Newcastle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Rain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">diff_city</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather Adjusted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wests tigers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dolphins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campbelltown Sports Stadium, Sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast titans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">penrith panthers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cbus Super Stadium, Gold Coast</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">canterbury-bankstown bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">manly-warringah sea eagles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accor Stadium, Sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">same_city_different_ground</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">warriors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north queensland cowboys</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One NZ Stadium, Christchurch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne storm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">canberra raiders</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AAMI Park, Melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney roosters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cronulla-sutherland sharks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allianz Stadium, Sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parramatta eels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">south sydney rabbitohs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CommBank Stadium, Sydney</t>
   </si>
 </sst>
 </file>
@@ -547,10 +553,10 @@
   <cols>
     <col min="1" max="1" width="4.9975" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="4.9975" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="25.5775" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="23.8625" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="23.005" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="25.5775" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.43" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="30.7225" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="37.5825" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="11.8575" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="14.43" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="14.43" hidden="0" customWidth="1"/>
@@ -569,6 +575,9 @@
     <col min="22" max="22" width="16.145" hidden="0" customWidth="1"/>
     <col min="23" max="23" width="16.145" hidden="0" customWidth="1"/>
     <col min="24" max="24" width="12.715" hidden="0" customWidth="1"/>
+    <col min="25" max="25" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="26" max="26" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="27" max="27" width="15.2875" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -644,31 +653,40 @@
       <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46192</v>
+        <v>46198</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0</v>
+        <v>5.27</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I2" s="5" t="n">
         <v>1</v>
@@ -677,72 +695,81 @@
         <v>1</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>-10.5</v>
+        <v>6.5</v>
       </c>
       <c r="L2" s="4" t="n">
         <v>49</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>-6.72</v>
+        <v>1.06</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>49.69</v>
+        <v>50.41</v>
       </c>
       <c r="O2" s="4" t="n">
-        <v>-11.85</v>
+        <v>0.1</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>50.01</v>
+        <v>47.46</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="R2" s="4" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.07</v>
+        <v>-0.01</v>
       </c>
       <c r="T2" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U2" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>-0.63</v>
+        <v>-0.3</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X2" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="Z2" s="4" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AA2" s="4" t="n">
+        <v>2.03</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46192</v>
+        <v>46198</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0</v>
+        <v>5.27</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>1</v>
@@ -751,73 +778,82 @@
         <v>1</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>-10.5</v>
+        <v>6.5</v>
       </c>
       <c r="L3" s="4" t="n">
         <v>49</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>-6.72</v>
+        <v>1.3</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>49.69</v>
+        <v>47.09</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>-11.85</v>
+        <v>0.1</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>50.01</v>
+        <v>47.46</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="R3" s="4" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.07</v>
+        <v>-0.01</v>
       </c>
       <c r="T3" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0</v>
+        <v>-0.24</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>-0.63</v>
+        <v>-0.3</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X3" s="4" t="n">
-        <v>0</v>
+        <v>-3.32</v>
+      </c>
+      <c r="Y3" s="4" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="Z3" s="4" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AA3" s="4" t="n">
+        <v>2.03</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46192</v>
+        <v>46198</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0</v>
+        <v>5.27</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>29</v>
-      </c>
       <c r="I4" s="5" t="n">
         <v>1</v>
       </c>
@@ -825,72 +861,81 @@
         <v>1</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>-10.5</v>
+        <v>6.5</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>49</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>-3.36</v>
+        <v>0.53</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>24.84</v>
+        <v>25.2</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>-5.93</v>
+        <v>0.05</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>25</v>
+        <v>23.73</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>1.25</v>
+        <v>0.5</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>-0.31</v>
+        <v>-0.15</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X4" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="Z4" s="4" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AA4" s="4" t="n">
+        <v>2.03</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46192</v>
+        <v>46198</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0</v>
+        <v>5.27</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>1</v>
@@ -899,72 +944,81 @@
         <v>1</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>-10.5</v>
+        <v>6.5</v>
       </c>
       <c r="L5" s="4" t="n">
         <v>49</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>-3.36</v>
+        <v>0.65</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>24.84</v>
+        <v>23.54</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>-5.93</v>
+        <v>0.05</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>25</v>
+        <v>23.73</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>1.25</v>
+        <v>0.5</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="T5" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>0</v>
+        <v>-0.12</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>-0.31</v>
+        <v>-0.15</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X5" s="4" t="n">
-        <v>0</v>
+        <v>-1.66</v>
+      </c>
+      <c r="Y5" s="4" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="Z5" s="4" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AA5" s="4" t="n">
+        <v>2.03</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0</v>
+        <v>3.97</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>1</v>
@@ -973,73 +1027,82 @@
         <v>1</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>8.5</v>
+        <v>1</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>52</v>
+        <v>46.5</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>-5.4</v>
+        <v>-4.98</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>53.13</v>
+        <v>50.6</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>-4.52</v>
+        <v>-7.44</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>53.45</v>
+        <v>48.03</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>-0.25</v>
+        <v>0.01</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>2.31</v>
+        <v>0</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X6" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y6" s="4" t="n">
+        <v>-0.91</v>
+      </c>
+      <c r="Z6" s="4" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="AA6" s="4" t="n">
+        <v>2.81</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="I7" s="5" t="n">
         <v>1</v>
       </c>
@@ -1047,73 +1110,82 @@
         <v>1</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>8.5</v>
+        <v>1</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>52</v>
+        <v>46.5</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>-5.4</v>
+        <v>-4.81</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>53.13</v>
+        <v>47.67</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>-4.52</v>
+        <v>-7.44</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>53.45</v>
+        <v>48.03</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R7" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>-0.25</v>
+        <v>0.01</v>
       </c>
       <c r="T7" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0</v>
+        <v>-0.17</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>2.31</v>
+        <v>0</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X7" s="4" t="n">
-        <v>0</v>
+        <v>-2.93</v>
+      </c>
+      <c r="Y7" s="4" t="n">
+        <v>-0.91</v>
+      </c>
+      <c r="Z7" s="4" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="AA7" s="4" t="n">
+        <v>2.81</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>29</v>
-      </c>
       <c r="I8" s="5" t="n">
         <v>1</v>
       </c>
@@ -1121,73 +1193,82 @@
         <v>1</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>8.5</v>
+        <v>1</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>52</v>
+        <v>46.5</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>-2.7</v>
+        <v>-2.49</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>26.57</v>
+        <v>25.3</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>-2.26</v>
+        <v>-3.72</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>26.72</v>
+        <v>24.01</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>1.25</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>-0.12</v>
+        <v>0.01</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>1.16</v>
+        <v>0</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X8" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y8" s="4" t="n">
+        <v>-0.91</v>
+      </c>
+      <c r="Z8" s="4" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="AA8" s="4" t="n">
+        <v>2.81</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="I9" s="5" t="n">
         <v>1</v>
       </c>
@@ -1195,72 +1276,81 @@
         <v>1</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>8.5</v>
+        <v>1</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>52</v>
+        <v>46.5</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>-2.7</v>
+        <v>-2.4</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>26.57</v>
+        <v>23.84</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>-2.26</v>
+        <v>-3.72</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>26.72</v>
+        <v>24.01</v>
       </c>
       <c r="Q9" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R9" s="4" t="n">
         <v>1.25</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>-0.12</v>
+        <v>0.01</v>
       </c>
       <c r="T9" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>0</v>
+        <v>-0.09</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.16</v>
+        <v>0</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X9" s="4" t="n">
-        <v>0</v>
+        <v>-1.46</v>
+      </c>
+      <c r="Y9" s="4" t="n">
+        <v>-0.91</v>
+      </c>
+      <c r="Z9" s="4" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="AA9" s="4" t="n">
+        <v>2.81</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>1</v>
@@ -1269,72 +1359,81 @@
         <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>12.5</v>
+        <v>3.5</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>49.5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>-1.79</v>
+        <v>-0.95</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>52.78</v>
+        <v>49.84</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>-1.58</v>
+        <v>-6.73</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>53.06</v>
+        <v>49.48</v>
       </c>
       <c r="Q10" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>-0.18</v>
+        <v>-0.02</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1.65</v>
+        <v>-0.63</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X10" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y10" s="4" t="n">
+        <v>-28.11</v>
+      </c>
+      <c r="Z10" s="4" t="n">
+        <v>-14.26</v>
+      </c>
+      <c r="AA10" s="4" t="n">
+        <v>-11.08</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>1</v>
@@ -1343,73 +1442,82 @@
         <v>1</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>12.5</v>
+        <v>3.5</v>
       </c>
       <c r="L11" s="4" t="n">
         <v>49.5</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>-1.79</v>
+        <v>-0.93</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>52.78</v>
+        <v>48.87</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>-1.58</v>
+        <v>-6.73</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>53.06</v>
+        <v>49.48</v>
       </c>
       <c r="Q11" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R11" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>-0.18</v>
+        <v>-0.02</v>
       </c>
       <c r="T11" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>1.65</v>
+        <v>-0.63</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X11" s="4" t="n">
-        <v>0</v>
+        <v>-0.98</v>
+      </c>
+      <c r="Y11" s="4" t="n">
+        <v>-28.11</v>
+      </c>
+      <c r="Z11" s="4" t="n">
+        <v>-14.26</v>
+      </c>
+      <c r="AA11" s="4" t="n">
+        <v>-11.08</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H12" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H12" s="3" t="s">
-        <v>29</v>
-      </c>
       <c r="I12" s="5" t="n">
         <v>1</v>
       </c>
@@ -1417,72 +1525,81 @@
         <v>1</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>12.5</v>
+        <v>3.5</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>49.5</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>-0.9</v>
+        <v>-0.48</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>26.39</v>
+        <v>24.92</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>-0.79</v>
+        <v>-3.36</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>26.53</v>
+        <v>24.74</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>1.25</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>-0.09</v>
+        <v>-0.01</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.83</v>
+        <v>-0.31</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X12" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y12" s="4" t="n">
+        <v>-28.11</v>
+      </c>
+      <c r="Z12" s="4" t="n">
+        <v>-14.26</v>
+      </c>
+      <c r="AA12" s="4" t="n">
+        <v>-11.08</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>1</v>
@@ -1491,72 +1608,81 @@
         <v>1</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>12.5</v>
+        <v>3.5</v>
       </c>
       <c r="L13" s="4" t="n">
         <v>49.5</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>-0.9</v>
+        <v>-0.47</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>26.39</v>
+        <v>24.43</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>-0.79</v>
+        <v>-3.36</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>26.53</v>
+        <v>24.74</v>
       </c>
       <c r="Q13" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R13" s="4" t="n">
         <v>1.25</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.09</v>
+        <v>-0.01</v>
       </c>
       <c r="T13" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>0.83</v>
+        <v>-0.31</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X13" s="4" t="n">
-        <v>0</v>
+        <v>-0.49</v>
+      </c>
+      <c r="Y13" s="4" t="n">
+        <v>-28.11</v>
+      </c>
+      <c r="Z13" s="4" t="n">
+        <v>-14.26</v>
+      </c>
+      <c r="AA13" s="4" t="n">
+        <v>-11.08</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46193</v>
+        <v>46200</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0</v>
+        <v>1.13</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>44</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>1</v>
@@ -1565,72 +1691,81 @@
         <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>7.5</v>
+        <v>-4</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>48.5</v>
+        <v>50.5</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>0.4</v>
+        <v>-7.17</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>50.42</v>
+        <v>52.55</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>1.88</v>
+        <v>-4.51</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>50.59</v>
+        <v>51.48</v>
       </c>
       <c r="Q14" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.04</v>
+        <v>-0.12</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>-0.32</v>
+        <v>2.29</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X14" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y14" s="4" t="n">
+        <v>21.73</v>
+      </c>
+      <c r="Z14" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="AA14" s="4" t="n">
+        <v>8.27</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46193</v>
+        <v>46200</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0</v>
+        <v>1.13</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>44</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>1</v>
@@ -1639,73 +1774,82 @@
         <v>1</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>7.5</v>
+        <v>-4</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>48.5</v>
+        <v>50.5</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.4</v>
+        <v>-7.12</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>50.42</v>
+        <v>51.08</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>1.88</v>
+        <v>-4.51</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>50.59</v>
+        <v>51.48</v>
       </c>
       <c r="Q15" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.04</v>
+        <v>-0.12</v>
       </c>
       <c r="T15" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0</v>
+        <v>-0.04</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>-0.32</v>
+        <v>2.29</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X15" s="4" t="n">
-        <v>0</v>
+        <v>-1.47</v>
+      </c>
+      <c r="Y15" s="4" t="n">
+        <v>21.73</v>
+      </c>
+      <c r="Z15" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="AA15" s="4" t="n">
+        <v>8.27</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46193</v>
+        <v>46200</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0</v>
+        <v>1.13</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>44</v>
       </c>
       <c r="G16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="3" t="s">
-        <v>29</v>
-      </c>
       <c r="I16" s="5" t="n">
         <v>1</v>
       </c>
@@ -1713,72 +1857,81 @@
         <v>1</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>7.5</v>
+        <v>-4</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>48.5</v>
+        <v>50.5</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>0.2</v>
+        <v>-3.58</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>25.21</v>
+        <v>26.28</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>0.94</v>
+        <v>-2.25</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>25.3</v>
+        <v>25.74</v>
       </c>
       <c r="Q16" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.02</v>
+        <v>-0.06</v>
       </c>
       <c r="T16" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>-0.16</v>
+        <v>1.14</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X16" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y16" s="4" t="n">
+        <v>21.73</v>
+      </c>
+      <c r="Z16" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="AA16" s="4" t="n">
+        <v>8.27</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46193</v>
+        <v>46200</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0</v>
+        <v>1.13</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>44</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>1</v>
@@ -1787,72 +1940,81 @@
         <v>1</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>7.5</v>
+        <v>-4</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>48.5</v>
+        <v>50.5</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>0.2</v>
+        <v>-3.56</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>25.21</v>
+        <v>25.54</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>0.94</v>
+        <v>-2.25</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>25.3</v>
+        <v>25.74</v>
       </c>
       <c r="Q17" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R17" s="4" t="n">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.02</v>
+        <v>-0.06</v>
       </c>
       <c r="T17" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>-0.16</v>
+        <v>1.14</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X17" s="4" t="n">
-        <v>0</v>
+        <v>-0.74</v>
+      </c>
+      <c r="Y17" s="4" t="n">
+        <v>21.73</v>
+      </c>
+      <c r="Z17" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="AA17" s="4" t="n">
+        <v>8.27</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46194</v>
+        <v>46200</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I18" s="5" t="n">
         <v>1</v>
@@ -1861,72 +2023,81 @@
         <v>1</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>-10</v>
+        <v>11.5</v>
       </c>
       <c r="L18" s="4" t="n">
         <v>50.5</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>9.87</v>
+        <v>-3.11</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>53.84</v>
+        <v>53.67</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>6.99</v>
+        <v>-7.2</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>53.45</v>
+        <v>52.87</v>
       </c>
       <c r="Q18" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R18" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>-0.28</v>
+        <v>-0.16</v>
       </c>
       <c r="T18" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>2.59</v>
+        <v>1.73</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X18" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y18" s="4" t="n">
+        <v>-4.02</v>
+      </c>
+      <c r="Z18" s="4" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="AA18" s="4" t="n">
+        <v>-11.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46194</v>
+        <v>46200</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>1</v>
@@ -1935,73 +2106,82 @@
         <v>1</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>-10</v>
+        <v>11.5</v>
       </c>
       <c r="L19" s="4" t="n">
         <v>50.5</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>9.9</v>
+        <v>-3.1</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>52.76</v>
+        <v>52.73</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>6.99</v>
+        <v>-7.2</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>53.45</v>
+        <v>52.87</v>
       </c>
       <c r="Q19" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R19" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>-0.28</v>
+        <v>-0.16</v>
       </c>
       <c r="T19" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>-0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>2.59</v>
+        <v>1.73</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X19" s="4" t="n">
-        <v>-1.08</v>
+        <v>-0.94</v>
+      </c>
+      <c r="Y19" s="4" t="n">
+        <v>-4.02</v>
+      </c>
+      <c r="Z19" s="4" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="AA19" s="4" t="n">
+        <v>-11.1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46194</v>
+        <v>46200</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G20" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H20" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H20" s="3" t="s">
-        <v>29</v>
-      </c>
       <c r="I20" s="5" t="n">
         <v>1</v>
       </c>
@@ -2009,72 +2189,81 @@
         <v>1</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>-10</v>
+        <v>11.5</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>50.5</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>4.94</v>
+        <v>-1.56</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>26.92</v>
+        <v>26.84</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>3.49</v>
+        <v>-3.6</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>26.72</v>
+        <v>26.44</v>
       </c>
       <c r="Q20" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>1.25</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>-0.14</v>
+        <v>-0.08</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>1.29</v>
+        <v>0.87</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X20" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y20" s="4" t="n">
+        <v>-4.02</v>
+      </c>
+      <c r="Z20" s="4" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="AA20" s="4" t="n">
+        <v>-11.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46194</v>
+        <v>46200</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I21" s="5" t="n">
         <v>1</v>
@@ -2083,72 +2272,81 @@
         <v>1</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>-10</v>
+        <v>11.5</v>
       </c>
       <c r="L21" s="4" t="n">
         <v>50.5</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>4.95</v>
+        <v>-1.55</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>26.38</v>
+        <v>26.36</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>3.49</v>
+        <v>-3.6</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>26.72</v>
+        <v>26.44</v>
       </c>
       <c r="Q21" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R21" s="4" t="n">
         <v>1.25</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>-0.14</v>
+        <v>-0.08</v>
       </c>
       <c r="T21" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U21" s="4" t="n">
         <v>-0.01</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>1.29</v>
+        <v>0.87</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X21" s="4" t="n">
-        <v>-0.54</v>
+        <v>-0.47</v>
+      </c>
+      <c r="Y21" s="4" t="n">
+        <v>-4.02</v>
+      </c>
+      <c r="Z21" s="4" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="AA21" s="4" t="n">
+        <v>-11.1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46194</v>
+        <v>46200</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>0.37</v>
+        <v>1.47</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I22" s="5" t="n">
         <v>1</v>
@@ -2157,72 +2355,81 @@
         <v>1</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>-9.5</v>
+        <v>-4.5</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>50.5</v>
+        <v>48</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>-6.41</v>
+        <v>-3.01</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>53.21</v>
+        <v>50.54</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>-1.88</v>
+        <v>-3.84</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>52.7</v>
+        <v>48.98</v>
       </c>
       <c r="Q22" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R22" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>-0.22</v>
+        <v>-0.01</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U22" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>1.97</v>
+        <v>-0.32</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X22" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y22" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="Z22" s="4" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="AA22" s="4" t="n">
+        <v>3.35</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46194</v>
+        <v>46200</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.37</v>
+        <v>1.47</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I23" s="5" t="n">
         <v>1</v>
@@ -2231,73 +2438,82 @@
         <v>1</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>-9.5</v>
+        <v>-4.5</v>
       </c>
       <c r="L23" s="4" t="n">
-        <v>50.5</v>
+        <v>48</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>-6.4</v>
+        <v>-2.95</v>
       </c>
       <c r="N23" s="4" t="n">
-        <v>52.58</v>
+        <v>48.87</v>
       </c>
       <c r="O23" s="4" t="n">
-        <v>-1.88</v>
+        <v>-3.84</v>
       </c>
       <c r="P23" s="4" t="n">
-        <v>52.7</v>
+        <v>48.98</v>
       </c>
       <c r="Q23" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R23" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>-0.22</v>
+        <v>-0.01</v>
       </c>
       <c r="T23" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>-0.01</v>
+        <v>-0.06</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>1.97</v>
+        <v>-0.32</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X23" s="4" t="n">
-        <v>-0.63</v>
+        <v>-1.67</v>
+      </c>
+      <c r="Y23" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="Z23" s="4" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="AA23" s="4" t="n">
+        <v>3.35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46194</v>
+        <v>46200</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0.37</v>
+        <v>1.47</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G24" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H24" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H24" s="3" t="s">
-        <v>29</v>
-      </c>
       <c r="I24" s="5" t="n">
         <v>1</v>
       </c>
@@ -2305,72 +2521,81 @@
         <v>1</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>-9.5</v>
+        <v>-4.5</v>
       </c>
       <c r="L24" s="4" t="n">
-        <v>50.5</v>
+        <v>48</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>-3.21</v>
+        <v>-1.51</v>
       </c>
       <c r="N24" s="4" t="n">
-        <v>26.6</v>
+        <v>25.27</v>
       </c>
       <c r="O24" s="4" t="n">
-        <v>-0.94</v>
+        <v>-1.92</v>
       </c>
       <c r="P24" s="4" t="n">
-        <v>26.35</v>
+        <v>24.49</v>
       </c>
       <c r="Q24" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R24" s="4" t="n">
         <v>1.25</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.11</v>
+        <v>0</v>
       </c>
       <c r="T24" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U24" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.99</v>
+        <v>-0.16</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X24" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y24" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="Z24" s="4" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="AA24" s="4" t="n">
+        <v>3.35</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46194</v>
+        <v>46200</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0.37</v>
+        <v>1.47</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I25" s="5" t="n">
         <v>1</v>
@@ -2379,72 +2604,81 @@
         <v>1</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>-9.5</v>
+        <v>-4.5</v>
       </c>
       <c r="L25" s="4" t="n">
-        <v>50.5</v>
+        <v>48</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>-3.2</v>
+        <v>-1.48</v>
       </c>
       <c r="N25" s="4" t="n">
-        <v>26.29</v>
+        <v>24.44</v>
       </c>
       <c r="O25" s="4" t="n">
-        <v>-0.94</v>
+        <v>-1.92</v>
       </c>
       <c r="P25" s="4" t="n">
-        <v>26.35</v>
+        <v>24.49</v>
       </c>
       <c r="Q25" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R25" s="4" t="n">
         <v>1.25</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.11</v>
+        <v>0</v>
       </c>
       <c r="T25" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>-0.01</v>
+        <v>-0.03</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>0.99</v>
+        <v>-0.16</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X25" s="4" t="n">
-        <v>-0.32</v>
+        <v>-0.84</v>
+      </c>
+      <c r="Y25" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="Z25" s="4" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="AA25" s="4" t="n">
+        <v>3.35</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46194</v>
+        <v>46201</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>1.8</v>
+        <v>1.33</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I26" s="5" t="n">
         <v>1</v>
@@ -2453,72 +2687,81 @@
         <v>1</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>-6</v>
+        <v>-11</v>
       </c>
       <c r="L26" s="4" t="n">
-        <v>50</v>
+        <v>52.5</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>-2.4</v>
+        <v>-5.43</v>
       </c>
       <c r="N26" s="4" t="n">
-        <v>50.7</v>
+        <v>53.2</v>
       </c>
       <c r="O26" s="4" t="n">
-        <v>-0.23</v>
+        <v>-10.37</v>
       </c>
       <c r="P26" s="4" t="n">
-        <v>49.15</v>
+        <v>51.72</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R26" s="4" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="T26" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U26" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0</v>
+        <v>2.64</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X26" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y26" s="4" t="n">
+        <v>-4.29</v>
+      </c>
+      <c r="Z26" s="4" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="AA26" s="4" t="n">
+        <v>-5.48</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46194</v>
+        <v>46201</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>1.8</v>
+        <v>1.33</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I27" s="5" t="n">
         <v>1</v>
@@ -2527,73 +2770,82 @@
         <v>1</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>-6</v>
+        <v>-11</v>
       </c>
       <c r="L27" s="4" t="n">
-        <v>50</v>
+        <v>52.5</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>-2.32</v>
+        <v>-5.38</v>
       </c>
       <c r="N27" s="4" t="n">
-        <v>48.76</v>
+        <v>51.54</v>
       </c>
       <c r="O27" s="4" t="n">
-        <v>-0.23</v>
+        <v>-10.37</v>
       </c>
       <c r="P27" s="4" t="n">
-        <v>49.15</v>
+        <v>51.72</v>
       </c>
       <c r="Q27" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="T27" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>-0.08</v>
+        <v>-0.05</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0</v>
+        <v>2.64</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X27" s="4" t="n">
-        <v>-1.93</v>
+        <v>-1.67</v>
+      </c>
+      <c r="Y27" s="4" t="n">
+        <v>-4.29</v>
+      </c>
+      <c r="Z27" s="4" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="AA27" s="4" t="n">
+        <v>-5.48</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46194</v>
+        <v>46201</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>1.8</v>
+        <v>1.33</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G28" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H28" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H28" s="3" t="s">
-        <v>29</v>
-      </c>
       <c r="I28" s="5" t="n">
         <v>1</v>
       </c>
@@ -2601,72 +2853,81 @@
         <v>1</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>-6</v>
+        <v>-11</v>
       </c>
       <c r="L28" s="4" t="n">
-        <v>50</v>
+        <v>52.5</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>-1.2</v>
+        <v>-2.72</v>
       </c>
       <c r="N28" s="4" t="n">
-        <v>25.35</v>
+        <v>26.6</v>
       </c>
       <c r="O28" s="4" t="n">
-        <v>-0.11</v>
+        <v>-5.19</v>
       </c>
       <c r="P28" s="4" t="n">
-        <v>24.58</v>
+        <v>25.86</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R28" s="4" t="n">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="T28" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U28" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>0</v>
+        <v>1.32</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X28" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y28" s="4" t="n">
+        <v>-4.29</v>
+      </c>
+      <c r="Z28" s="4" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="AA28" s="4" t="n">
+        <v>-5.48</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46194</v>
+        <v>46201</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>1.8</v>
+        <v>1.33</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I29" s="5" t="n">
         <v>1</v>
@@ -2675,326 +2936,387 @@
         <v>1</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>-6</v>
+        <v>-11</v>
       </c>
       <c r="L29" s="4" t="n">
-        <v>50</v>
+        <v>52.5</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>-1.16</v>
+        <v>-2.69</v>
       </c>
       <c r="N29" s="4" t="n">
-        <v>24.38</v>
+        <v>25.77</v>
       </c>
       <c r="O29" s="4" t="n">
-        <v>-0.11</v>
+        <v>-5.19</v>
       </c>
       <c r="P29" s="4" t="n">
-        <v>24.58</v>
+        <v>25.86</v>
       </c>
       <c r="Q29" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R29" s="4" t="n">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="T29" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>-0.04</v>
+        <v>-0.03</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>0</v>
+        <v>1.32</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X29" s="4" t="n">
-        <v>-0.97</v>
+        <v>-0.83</v>
+      </c>
+      <c r="Y29" s="4" t="n">
+        <v>-4.29</v>
+      </c>
+      <c r="Z29" s="4" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="AA29" s="4" t="n">
+        <v>-5.48</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46198</v>
+        <v>46201</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="4"/>
-      <c r="L30" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="L30" s="4" t="n">
+        <v>52</v>
+      </c>
       <c r="M30" s="4" t="n">
-        <v>-0.08</v>
+        <v>-3.29</v>
       </c>
       <c r="N30" s="4" t="n">
-        <v>50.91</v>
+        <v>53.32</v>
       </c>
       <c r="O30" s="4" t="n">
-        <v>-0.09</v>
+        <v>-4.78</v>
       </c>
       <c r="P30" s="4" t="n">
-        <v>50.91</v>
+        <v>52.98</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R30" s="4" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.04</v>
+        <v>-0.14</v>
       </c>
       <c r="T30" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U30" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>-0.32</v>
+        <v>2.04</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X30" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y30" s="4" t="n">
+        <v>13.92</v>
+      </c>
+      <c r="Z30" s="4" t="n">
+        <v>-19.15</v>
+      </c>
+      <c r="AA30" s="4" t="n">
+        <v>26.46</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46198</v>
+        <v>46201</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="4"/>
-      <c r="L31" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="K31" s="4" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="L31" s="4" t="n">
+        <v>52</v>
+      </c>
       <c r="M31" s="4" t="n">
-        <v>-0.08</v>
+        <v>-3.28</v>
       </c>
       <c r="N31" s="4" t="n">
-        <v>50.91</v>
+        <v>52.51</v>
       </c>
       <c r="O31" s="4" t="n">
-        <v>-0.09</v>
+        <v>-4.78</v>
       </c>
       <c r="P31" s="4" t="n">
-        <v>50.91</v>
+        <v>52.98</v>
       </c>
       <c r="Q31" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R31" s="4" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.04</v>
+        <v>-0.14</v>
       </c>
       <c r="T31" s="4" t="n">
-        <v>-1.92</v>
+        <v>-1.87</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.32</v>
+        <v>2.04</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>4.02</v>
       </c>
       <c r="X31" s="4" t="n">
-        <v>0</v>
+        <v>-0.81</v>
+      </c>
+      <c r="Y31" s="4" t="n">
+        <v>13.92</v>
+      </c>
+      <c r="Z31" s="4" t="n">
+        <v>-19.15</v>
+      </c>
+      <c r="AA31" s="4" t="n">
+        <v>26.46</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46198</v>
+        <v>46201</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G32" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H32" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H32" s="3" t="s">
-        <v>29</v>
-      </c>
       <c r="I32" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" s="4"/>
-      <c r="L32" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>52</v>
+      </c>
       <c r="M32" s="4" t="n">
-        <v>-0.04</v>
+        <v>-1.65</v>
       </c>
       <c r="N32" s="4" t="n">
-        <v>25.46</v>
+        <v>26.66</v>
       </c>
       <c r="O32" s="4" t="n">
-        <v>-0.04</v>
+        <v>-2.39</v>
       </c>
       <c r="P32" s="4" t="n">
-        <v>25.46</v>
+        <v>26.49</v>
       </c>
       <c r="Q32" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R32" s="4" t="n">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.02</v>
+        <v>-0.07</v>
       </c>
       <c r="T32" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U32" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>-0.16</v>
+        <v>1.02</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X32" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="Y32" s="4" t="n">
+        <v>13.92</v>
+      </c>
+      <c r="Z32" s="4" t="n">
+        <v>-19.15</v>
+      </c>
+      <c r="AA32" s="4" t="n">
+        <v>26.46</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46198</v>
+        <v>46201</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="L33" s="4" t="n">
+        <v>52</v>
+      </c>
       <c r="M33" s="4" t="n">
-        <v>-0.04</v>
+        <v>-1.64</v>
       </c>
       <c r="N33" s="4" t="n">
-        <v>25.46</v>
+        <v>26.26</v>
       </c>
       <c r="O33" s="4" t="n">
-        <v>-0.04</v>
+        <v>-2.39</v>
       </c>
       <c r="P33" s="4" t="n">
-        <v>25.46</v>
+        <v>26.49</v>
       </c>
       <c r="Q33" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="R33" s="4" t="n">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="S33" s="4" t="n">
-        <v>0.02</v>
+        <v>-0.07</v>
       </c>
       <c r="T33" s="4" t="n">
-        <v>-0.96</v>
+        <v>-0.94</v>
       </c>
       <c r="U33" s="4" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="V33" s="4" t="n">
-        <v>-0.16</v>
+        <v>1.02</v>
       </c>
       <c r="W33" s="4" t="n">
         <v>2.01</v>
       </c>
       <c r="X33" s="4" t="n">
-        <v>0</v>
+        <v>-0.4</v>
+      </c>
+      <c r="Y33" s="4" t="n">
+        <v>13.92</v>
+      </c>
+      <c r="Z33" s="4" t="n">
+        <v>-19.15</v>
+      </c>
+      <c r="AA33" s="4" t="n">
+        <v>26.46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-08-01 08:45:33
</commit_message>
<xml_diff>
--- a/files/NRL_upcoming_projections.xlsx
+++ b/files/NRL_upcoming_projections.xlsx
@@ -572,12 +572,8 @@
       <c r="H2" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J2" t="n">
-        <v>49.5</v>
-      </c>
+      <c r="I2"/>
+      <c r="J2"/>
       <c r="K2" t="s">
         <v>17</v>
       </c>
@@ -610,12 +606,8 @@
       <c r="H3" t="s">
         <v>18</v>
       </c>
-      <c r="I3" t="n">
-        <v>10</v>
-      </c>
-      <c r="J3" t="n">
-        <v>49.5</v>
-      </c>
+      <c r="I3"/>
+      <c r="J3"/>
       <c r="K3" t="s">
         <v>17</v>
       </c>
@@ -648,12 +640,8 @@
       <c r="H4" t="s">
         <v>16</v>
       </c>
-      <c r="I4" t="n">
-        <v>10</v>
-      </c>
-      <c r="J4" t="n">
-        <v>49.5</v>
-      </c>
+      <c r="I4"/>
+      <c r="J4"/>
       <c r="K4" t="s">
         <v>17</v>
       </c>
@@ -686,12 +674,8 @@
       <c r="H5" t="s">
         <v>18</v>
       </c>
-      <c r="I5" t="n">
-        <v>10</v>
-      </c>
-      <c r="J5" t="n">
-        <v>49.5</v>
-      </c>
+      <c r="I5"/>
+      <c r="J5"/>
       <c r="K5" t="s">
         <v>17</v>
       </c>
@@ -861,7 +845,7 @@
         <v>16</v>
       </c>
       <c r="I10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10" t="n">
         <v>49.5</v>
@@ -899,7 +883,7 @@
         <v>18</v>
       </c>
       <c r="I11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J11" t="n">
         <v>49.5</v>
@@ -937,7 +921,7 @@
         <v>16</v>
       </c>
       <c r="I12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J12" t="n">
         <v>49.5</v>
@@ -975,7 +959,7 @@
         <v>18</v>
       </c>
       <c r="I13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13" t="n">
         <v>49.5</v>
@@ -1013,10 +997,10 @@
         <v>16</v>
       </c>
       <c r="I14" t="n">
-        <v>-10.5</v>
+        <v>-9</v>
       </c>
       <c r="J14" t="n">
-        <v>42.5</v>
+        <v>44</v>
       </c>
       <c r="K14" t="s">
         <v>31</v>
@@ -1051,10 +1035,10 @@
         <v>18</v>
       </c>
       <c r="I15" t="n">
-        <v>-10.5</v>
+        <v>-9</v>
       </c>
       <c r="J15" t="n">
-        <v>42.5</v>
+        <v>44</v>
       </c>
       <c r="K15" t="s">
         <v>31</v>
@@ -1089,10 +1073,10 @@
         <v>16</v>
       </c>
       <c r="I16" t="n">
-        <v>-10.5</v>
+        <v>-9</v>
       </c>
       <c r="J16" t="n">
-        <v>42.5</v>
+        <v>44</v>
       </c>
       <c r="K16" t="s">
         <v>31</v>
@@ -1127,10 +1111,10 @@
         <v>18</v>
       </c>
       <c r="I17" t="n">
-        <v>-10.5</v>
+        <v>-9</v>
       </c>
       <c r="J17" t="n">
-        <v>42.5</v>
+        <v>44</v>
       </c>
       <c r="K17" t="s">
         <v>31</v>
@@ -1164,8 +1148,12 @@
       <c r="H18" t="s">
         <v>16</v>
       </c>
-      <c r="I18"/>
-      <c r="J18"/>
+      <c r="I18" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="J18" t="n">
+        <v>46</v>
+      </c>
       <c r="K18" t="s">
         <v>35</v>
       </c>
@@ -1198,8 +1186,12 @@
       <c r="H19" t="s">
         <v>18</v>
       </c>
-      <c r="I19"/>
-      <c r="J19"/>
+      <c r="I19" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="J19" t="n">
+        <v>46</v>
+      </c>
       <c r="K19" t="s">
         <v>35</v>
       </c>
@@ -1232,8 +1224,12 @@
       <c r="H20" t="s">
         <v>16</v>
       </c>
-      <c r="I20"/>
-      <c r="J20"/>
+      <c r="I20" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="J20" t="n">
+        <v>46</v>
+      </c>
       <c r="K20" t="s">
         <v>35</v>
       </c>
@@ -1266,8 +1262,12 @@
       <c r="H21" t="s">
         <v>18</v>
       </c>
-      <c r="I21"/>
-      <c r="J21"/>
+      <c r="I21" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>46</v>
+      </c>
       <c r="K21" t="s">
         <v>35</v>
       </c>
@@ -1301,10 +1301,10 @@
         <v>16</v>
       </c>
       <c r="I22" t="n">
-        <v>-7.5</v>
+        <v>-12.5</v>
       </c>
       <c r="J22" t="n">
-        <v>48.5</v>
+        <v>52</v>
       </c>
       <c r="K22" t="s">
         <v>39</v>
@@ -1339,10 +1339,10 @@
         <v>18</v>
       </c>
       <c r="I23" t="n">
-        <v>-7.5</v>
+        <v>-12.5</v>
       </c>
       <c r="J23" t="n">
-        <v>48.5</v>
+        <v>52</v>
       </c>
       <c r="K23" t="s">
         <v>39</v>
@@ -1377,10 +1377,10 @@
         <v>16</v>
       </c>
       <c r="I24" t="n">
-        <v>-7.5</v>
+        <v>-12.5</v>
       </c>
       <c r="J24" t="n">
-        <v>48.5</v>
+        <v>52</v>
       </c>
       <c r="K24" t="s">
         <v>39</v>
@@ -1415,10 +1415,10 @@
         <v>18</v>
       </c>
       <c r="I25" t="n">
-        <v>-7.5</v>
+        <v>-12.5</v>
       </c>
       <c r="J25" t="n">
-        <v>48.5</v>
+        <v>52</v>
       </c>
       <c r="K25" t="s">
         <v>39</v>
@@ -1453,10 +1453,10 @@
         <v>16</v>
       </c>
       <c r="I26" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="J26" t="n">
-        <v>48.5</v>
+        <v>49</v>
       </c>
       <c r="K26" t="s">
         <v>43</v>
@@ -1491,10 +1491,10 @@
         <v>18</v>
       </c>
       <c r="I27" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="J27" t="n">
-        <v>48.5</v>
+        <v>49</v>
       </c>
       <c r="K27" t="s">
         <v>43</v>
@@ -1529,10 +1529,10 @@
         <v>16</v>
       </c>
       <c r="I28" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="J28" t="n">
-        <v>48.5</v>
+        <v>49</v>
       </c>
       <c r="K28" t="s">
         <v>43</v>
@@ -1567,10 +1567,10 @@
         <v>18</v>
       </c>
       <c r="I29" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="J29" t="n">
-        <v>48.5</v>
+        <v>49</v>
       </c>
       <c r="K29" t="s">
         <v>43</v>
@@ -1604,8 +1604,12 @@
       <c r="H30" t="s">
         <v>16</v>
       </c>
-      <c r="I30"/>
-      <c r="J30"/>
+      <c r="I30" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J30" t="n">
+        <v>47.5</v>
+      </c>
       <c r="K30" t="s">
         <v>27</v>
       </c>
@@ -1638,8 +1642,12 @@
       <c r="H31" t="s">
         <v>18</v>
       </c>
-      <c r="I31"/>
-      <c r="J31"/>
+      <c r="I31" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J31" t="n">
+        <v>47.5</v>
+      </c>
       <c r="K31" t="s">
         <v>27</v>
       </c>
@@ -1672,8 +1680,12 @@
       <c r="H32" t="s">
         <v>16</v>
       </c>
-      <c r="I32"/>
-      <c r="J32"/>
+      <c r="I32" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J32" t="n">
+        <v>47.5</v>
+      </c>
       <c r="K32" t="s">
         <v>27</v>
       </c>
@@ -1706,8 +1718,12 @@
       <c r="H33" t="s">
         <v>18</v>
       </c>
-      <c r="I33"/>
-      <c r="J33"/>
+      <c r="I33" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J33" t="n">
+        <v>47.5</v>
+      </c>
       <c r="K33" t="s">
         <v>27</v>
       </c>
@@ -1740,8 +1756,12 @@
       <c r="H34" t="s">
         <v>16</v>
       </c>
-      <c r="I34"/>
-      <c r="J34"/>
+      <c r="I34" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="J34" t="n">
+        <v>45.5</v>
+      </c>
       <c r="K34" t="s">
         <v>47</v>
       </c>
@@ -1774,8 +1794,12 @@
       <c r="H35" t="s">
         <v>18</v>
       </c>
-      <c r="I35"/>
-      <c r="J35"/>
+      <c r="I35" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="J35" t="n">
+        <v>45.5</v>
+      </c>
       <c r="K35" t="s">
         <v>47</v>
       </c>
@@ -1808,8 +1832,12 @@
       <c r="H36" t="s">
         <v>16</v>
       </c>
-      <c r="I36"/>
-      <c r="J36"/>
+      <c r="I36" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="J36" t="n">
+        <v>45.5</v>
+      </c>
       <c r="K36" t="s">
         <v>47</v>
       </c>
@@ -1842,8 +1870,12 @@
       <c r="H37" t="s">
         <v>18</v>
       </c>
-      <c r="I37"/>
-      <c r="J37"/>
+      <c r="I37" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="J37" t="n">
+        <v>45.5</v>
+      </c>
       <c r="K37" t="s">
         <v>47</v>
       </c>
@@ -1876,8 +1908,12 @@
       <c r="H38" t="s">
         <v>16</v>
       </c>
-      <c r="I38"/>
-      <c r="J38"/>
+      <c r="I38" t="n">
+        <v>5</v>
+      </c>
+      <c r="J38" t="n">
+        <v>40.5</v>
+      </c>
       <c r="K38" t="s">
         <v>48</v>
       </c>
@@ -1910,8 +1946,12 @@
       <c r="H39" t="s">
         <v>18</v>
       </c>
-      <c r="I39"/>
-      <c r="J39"/>
+      <c r="I39" t="n">
+        <v>5</v>
+      </c>
+      <c r="J39" t="n">
+        <v>40.5</v>
+      </c>
       <c r="K39" t="s">
         <v>48</v>
       </c>
@@ -1944,8 +1984,12 @@
       <c r="H40" t="s">
         <v>16</v>
       </c>
-      <c r="I40"/>
-      <c r="J40"/>
+      <c r="I40" t="n">
+        <v>5</v>
+      </c>
+      <c r="J40" t="n">
+        <v>40.5</v>
+      </c>
       <c r="K40" t="s">
         <v>48</v>
       </c>
@@ -1978,8 +2022,12 @@
       <c r="H41" t="s">
         <v>18</v>
       </c>
-      <c r="I41"/>
-      <c r="J41"/>
+      <c r="I41" t="n">
+        <v>5</v>
+      </c>
+      <c r="J41" t="n">
+        <v>40.5</v>
+      </c>
       <c r="K41" t="s">
         <v>48</v>
       </c>

</xml_diff>

<commit_message>
Update model outputs 2026-08-03 20:19:43
</commit_message>
<xml_diff>
--- a/files/NRL_upcoming_projections.xlsx
+++ b/files/NRL_upcoming_projections.xlsx
@@ -561,7 +561,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>-8.1</v>
+        <v>-5.3</v>
       </c>
       <c r="F2" t="n">
         <v>46</v>
@@ -599,7 +599,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>-8.1</v>
+        <v>-5.3</v>
       </c>
       <c r="F3" t="n">
         <v>46</v>
@@ -637,7 +637,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>-4</v>
+        <v>-2.7</v>
       </c>
       <c r="F4" t="n">
         <v>23</v>
@@ -675,7 +675,7 @@
         <v>14</v>
       </c>
       <c r="E5" t="n">
-        <v>-4</v>
+        <v>-2.7</v>
       </c>
       <c r="F5" t="n">
         <v>23</v>
@@ -713,7 +713,7 @@
         <v>22</v>
       </c>
       <c r="E6" t="n">
-        <v>3.1</v>
+        <v>3.9</v>
       </c>
       <c r="F6" t="n">
         <v>44.4</v>
@@ -751,7 +751,7 @@
         <v>22</v>
       </c>
       <c r="E7" t="n">
-        <v>3.1</v>
+        <v>3.9</v>
       </c>
       <c r="F7" t="n">
         <v>44.4</v>
@@ -789,7 +789,7 @@
         <v>22</v>
       </c>
       <c r="E8" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="F8" t="n">
         <v>22.2</v>
@@ -827,7 +827,7 @@
         <v>22</v>
       </c>
       <c r="E9" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="F9" t="n">
         <v>22.2</v>
@@ -865,7 +865,7 @@
         <v>26</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
         <v>45.7</v>
@@ -903,7 +903,7 @@
         <v>26</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
         <v>45.7</v>
@@ -941,7 +941,7 @@
         <v>26</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
         <v>22.9</v>
@@ -979,7 +979,7 @@
         <v>26</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
         <v>22.9</v>
@@ -1017,7 +1017,7 @@
         <v>30</v>
       </c>
       <c r="E14" t="n">
-        <v>-9.5</v>
+        <v>-8.1</v>
       </c>
       <c r="F14" t="n">
         <v>39.1</v>
@@ -1055,7 +1055,7 @@
         <v>30</v>
       </c>
       <c r="E15" t="n">
-        <v>-9.5</v>
+        <v>-8.1</v>
       </c>
       <c r="F15" t="n">
         <v>39.1</v>
@@ -1093,7 +1093,7 @@
         <v>30</v>
       </c>
       <c r="E16" t="n">
-        <v>-4.7</v>
+        <v>-4</v>
       </c>
       <c r="F16" t="n">
         <v>19.6</v>
@@ -1131,7 +1131,7 @@
         <v>30</v>
       </c>
       <c r="E17" t="n">
-        <v>-4.7</v>
+        <v>-4</v>
       </c>
       <c r="F17" t="n">
         <v>19.6</v>
@@ -1169,7 +1169,7 @@
         <v>33</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="F18" t="n">
         <v>38.3</v>
@@ -1207,7 +1207,7 @@
         <v>33</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="F19" t="n">
         <v>38.3</v>
@@ -1245,7 +1245,7 @@
         <v>33</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F20" t="n">
         <v>19.2</v>
@@ -1283,7 +1283,7 @@
         <v>33</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F21" t="n">
         <v>19.2</v>
@@ -1321,7 +1321,7 @@
         <v>37</v>
       </c>
       <c r="E22" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="F22" t="n">
         <v>40.9</v>
@@ -1359,7 +1359,7 @@
         <v>37</v>
       </c>
       <c r="E23" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="F23" t="n">
         <v>40.5</v>
@@ -1397,7 +1397,7 @@
         <v>37</v>
       </c>
       <c r="E24" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
         <v>20.4</v>
@@ -1435,7 +1435,7 @@
         <v>37</v>
       </c>
       <c r="E25" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
         <v>20.3</v>
@@ -1473,7 +1473,7 @@
         <v>41</v>
       </c>
       <c r="E26" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="F26" t="n">
         <v>46.3</v>
@@ -1511,7 +1511,7 @@
         <v>41</v>
       </c>
       <c r="E27" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="F27" t="n">
         <v>46.3</v>
@@ -1549,7 +1549,7 @@
         <v>41</v>
       </c>
       <c r="E28" t="n">
-        <v>-2</v>
+        <v>-2.5</v>
       </c>
       <c r="F28" t="n">
         <v>23.1</v>
@@ -1587,7 +1587,7 @@
         <v>41</v>
       </c>
       <c r="E29" t="n">
-        <v>-2</v>
+        <v>-2.5</v>
       </c>
       <c r="F29" t="n">
         <v>23.1</v>
@@ -1625,7 +1625,7 @@
         <v>22</v>
       </c>
       <c r="E30" t="n">
-        <v>-3.4</v>
+        <v>-8</v>
       </c>
       <c r="F30" t="n">
         <v>46.3</v>
@@ -1663,7 +1663,7 @@
         <v>22</v>
       </c>
       <c r="E31" t="n">
-        <v>-3.4</v>
+        <v>-8</v>
       </c>
       <c r="F31" t="n">
         <v>46.1</v>
@@ -1701,7 +1701,7 @@
         <v>22</v>
       </c>
       <c r="E32" t="n">
-        <v>-1.7</v>
+        <v>-4</v>
       </c>
       <c r="F32" t="n">
         <v>23.1</v>
@@ -1739,7 +1739,7 @@
         <v>22</v>
       </c>
       <c r="E33" t="n">
-        <v>-1.7</v>
+        <v>-4</v>
       </c>
       <c r="F33" t="n">
         <v>23.1</v>
@@ -1777,7 +1777,7 @@
         <v>45</v>
       </c>
       <c r="E34" t="n">
-        <v>-1.9</v>
+        <v>-1.8</v>
       </c>
       <c r="F34" t="n">
         <v>44</v>
@@ -1815,7 +1815,7 @@
         <v>45</v>
       </c>
       <c r="E35" t="n">
-        <v>-1.9</v>
+        <v>-1.8</v>
       </c>
       <c r="F35" t="n">
         <v>41.6</v>
@@ -1929,7 +1929,7 @@
         <v>13</v>
       </c>
       <c r="E38" t="n">
-        <v>10.8</v>
+        <v>12.1</v>
       </c>
       <c r="F38" t="n">
         <v>42.6</v>
@@ -1967,7 +1967,7 @@
         <v>13</v>
       </c>
       <c r="E39" t="n">
-        <v>10.8</v>
+        <v>12.1</v>
       </c>
       <c r="F39" t="n">
         <v>41.7</v>
@@ -2005,7 +2005,7 @@
         <v>13</v>
       </c>
       <c r="E40" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="F40" t="n">
         <v>21.3</v>
@@ -2043,7 +2043,7 @@
         <v>13</v>
       </c>
       <c r="E41" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="F41" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
Update model outputs 2026-09-01 21:01:07
</commit_message>
<xml_diff>
--- a/files/NRL_upcoming_projections.xlsx
+++ b/files/NRL_upcoming_projections.xlsx
@@ -1819,7 +1819,7 @@
         <v>18</v>
       </c>
       <c r="K30" t="n">
-        <v>-19.5</v>
+        <v>-19</v>
       </c>
       <c r="L30" t="n">
         <v>48</v>
@@ -1863,7 +1863,7 @@
         <v>20</v>
       </c>
       <c r="K31" t="n">
-        <v>-19.5</v>
+        <v>-19</v>
       </c>
       <c r="L31" t="n">
         <v>48</v>
@@ -1907,7 +1907,7 @@
         <v>18</v>
       </c>
       <c r="K32" t="n">
-        <v>-19.5</v>
+        <v>-19</v>
       </c>
       <c r="L32" t="n">
         <v>48</v>
@@ -1951,7 +1951,7 @@
         <v>20</v>
       </c>
       <c r="K33" t="n">
-        <v>-19.5</v>
+        <v>-19</v>
       </c>
       <c r="L33" t="n">
         <v>48</v>

</xml_diff>